<commit_message>
Complete fixed-input cabling and verify continuous five-step engineering chain
</commit_message>
<xml_diff>
--- a/dev/backend/internal/engineering/testdata/five-step/03-cabling.xlsx
+++ b/dev/backend/internal/engineering/testdata/five-step/03-cabling.xlsx
@@ -160,7 +160,7 @@
     <t>引线规则引用</t>
   </si>
   <si>
-    <t>fixture-lead-2m-v1</t>
+    <t>fixture-lead-2m@1</t>
   </si>
   <si>
     <t>规格编码</t>
@@ -235,10 +235,10 @@
     <t>shortest_path</t>
   </si>
   <si>
-    <t>fixture-slack-10pct-v1</t>
-  </si>
-  <si>
-    <t>fixture-stock-ceiling-v1</t>
+    <t>fixture-slack-10pct@1</t>
+  </si>
+  <si>
+    <t>fixture-stock-ceiling@1</t>
   </si>
   <si>
     <t>SYNTHETIC_ONLY: rules must be explicitly created and approved in the test project</t>

</xml_diff>